<commit_message>
chi test is started
</commit_message>
<xml_diff>
--- a/Data/KW_dunn_results_withing_month.xlsx
+++ b/Data/KW_dunn_results_withing_month.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e91640961c0a8f3d/Рабочий стол/Python_repos/Python_projects_ICG_SB_RAS/Four_host_species_OF/Data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_6364C174AEB0F24CC888A89E23012B66ADA97C07" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liver_results" sheetId="1" r:id="rId1"/>
     <sheet name="Fluke_results" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -107,8 +113,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -198,13 +204,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -242,7 +256,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -276,6 +290,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -310,9 +325,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -485,11 +501,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -500,7 +516,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -511,7 +527,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -522,7 +538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
@@ -560,7 +576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -571,7 +587,7 @@
         <v>0.06</v>
       </c>
       <c r="D5" s="4">
-        <v>0.598</v>
+        <v>0.59799999999999998</v>
       </c>
       <c r="E5" s="4">
         <v>0.85</v>
@@ -583,13 +599,13 @@
         <v>1</v>
       </c>
       <c r="I5" s="4">
-        <v>0.8100000000000001</v>
+        <v>0.81</v>
       </c>
       <c r="J5" s="4">
         <v>0.314</v>
       </c>
       <c r="K5" s="4">
-        <v>0.119</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>0</v>
@@ -598,16 +614,16 @@
         <v>1</v>
       </c>
       <c r="O5" s="4">
-        <v>0.708</v>
+        <v>0.70799999999999996</v>
       </c>
       <c r="P5" s="4">
         <v>0.372</v>
       </c>
       <c r="Q5" s="5">
-        <v>0.042</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17">
+        <v>4.2000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
@@ -618,7 +634,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="4">
-        <v>0.197</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="E6" s="4">
         <v>0.06</v>
@@ -627,22 +643,22 @@
         <v>1</v>
       </c>
       <c r="H6" s="4">
-        <v>0.8100000000000001</v>
+        <v>0.81</v>
       </c>
       <c r="I6" s="4">
         <v>1</v>
       </c>
       <c r="J6" s="4">
-        <v>0.259</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="K6" s="4">
-        <v>0.138</v>
+        <v>0.13800000000000001</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="N6" s="4">
-        <v>0.708</v>
+        <v>0.70799999999999996</v>
       </c>
       <c r="O6" s="4">
         <v>1</v>
@@ -651,24 +667,24 @@
         <v>0.247</v>
       </c>
       <c r="Q6" s="4">
-        <v>0.074</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17">
+        <v>7.3999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="4">
-        <v>0.598</v>
+        <v>0.59799999999999998</v>
       </c>
       <c r="C7" s="4">
-        <v>0.197</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
       </c>
       <c r="E7" s="4">
-        <v>0.579</v>
+        <v>0.57899999999999996</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>2</v>
@@ -677,13 +693,13 @@
         <v>0.314</v>
       </c>
       <c r="I7" s="4">
-        <v>0.259</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="J7" s="4">
         <v>1</v>
       </c>
       <c r="K7" s="5">
-        <v>0.008999999999999999</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>2</v>
@@ -698,10 +714,10 @@
         <v>1</v>
       </c>
       <c r="Q7" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -712,7 +728,7 @@
         <v>0.06</v>
       </c>
       <c r="D8" s="4">
-        <v>0.579</v>
+        <v>0.57899999999999996</v>
       </c>
       <c r="E8" s="4">
         <v>1</v>
@@ -721,13 +737,13 @@
         <v>3</v>
       </c>
       <c r="H8" s="4">
-        <v>0.119</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="I8" s="4">
-        <v>0.138</v>
+        <v>0.13800000000000001</v>
       </c>
       <c r="J8" s="5">
-        <v>0.008999999999999999</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="K8" s="4">
         <v>1</v>
@@ -736,19 +752,19 @@
         <v>3</v>
       </c>
       <c r="N8" s="5">
-        <v>0.042</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="O8" s="4">
-        <v>0.074</v>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="P8" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="Q8" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -759,7 +775,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>7</v>
       </c>
@@ -770,7 +786,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -781,7 +797,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>0</v>
       </c>
@@ -819,7 +835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>0</v>
       </c>
@@ -827,13 +843,13 @@
         <v>1</v>
       </c>
       <c r="C15" s="4">
-        <v>0.909</v>
+        <v>0.90900000000000003</v>
       </c>
       <c r="D15" s="4">
-        <v>0.978</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="E15" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>0</v>
@@ -842,13 +858,13 @@
         <v>1</v>
       </c>
       <c r="I15" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="J15" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="K15" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>0</v>
@@ -857,121 +873,121 @@
         <v>1</v>
       </c>
       <c r="O15" s="4">
-        <v>0.574</v>
+        <v>0.57399999999999995</v>
       </c>
       <c r="P15" s="4">
-        <v>0.328</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="Q15" s="4">
-        <v>0.056</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17">
+        <v>5.6000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B16" s="4">
-        <v>0.909</v>
+        <v>0.90900000000000003</v>
       </c>
       <c r="C16" s="4">
         <v>1</v>
       </c>
       <c r="D16" s="4">
-        <v>0.909</v>
+        <v>0.90900000000000003</v>
       </c>
       <c r="E16" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="H16" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="I16" s="4">
         <v>1</v>
       </c>
       <c r="J16" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="K16" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="N16" s="4">
-        <v>0.574</v>
+        <v>0.57399999999999995</v>
       </c>
       <c r="O16" s="4">
         <v>1</v>
       </c>
       <c r="P16" s="4">
-        <v>0.146</v>
+        <v>0.14599999999999999</v>
       </c>
       <c r="Q16" s="4">
-        <v>0.146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
+        <v>0.14599999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B17" s="4">
-        <v>0.978</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="C17" s="4">
-        <v>0.909</v>
+        <v>0.90900000000000003</v>
       </c>
       <c r="D17" s="4">
         <v>1</v>
       </c>
       <c r="E17" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H17" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="I17" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="J17" s="4">
         <v>1</v>
       </c>
       <c r="K17" s="5">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="N17" s="4">
-        <v>0.328</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="O17" s="4">
-        <v>0.146</v>
+        <v>0.14599999999999999</v>
       </c>
       <c r="P17" s="4">
         <v>1</v>
       </c>
       <c r="Q17" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B18" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="C18" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="D18" s="4">
-        <v>0.599</v>
+        <v>0.59899999999999998</v>
       </c>
       <c r="E18" s="4">
         <v>1</v>
@@ -980,13 +996,13 @@
         <v>3</v>
       </c>
       <c r="H18" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I18" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="J18" s="5">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="K18" s="4">
         <v>1</v>
@@ -995,19 +1011,19 @@
         <v>3</v>
       </c>
       <c r="N18" s="4">
-        <v>0.056</v>
+        <v>5.6000000000000001E-2</v>
       </c>
       <c r="O18" s="4">
-        <v>0.146</v>
+        <v>0.14599999999999999</v>
       </c>
       <c r="P18" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="Q18" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1018,7 +1034,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>8</v>
       </c>
@@ -1029,7 +1045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -1040,7 +1056,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>0</v>
       </c>
@@ -1078,7 +1094,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>0</v>
       </c>
@@ -1086,13 +1102,13 @@
         <v>1</v>
       </c>
       <c r="C25" s="4">
-        <v>0.788</v>
+        <v>0.78800000000000003</v>
       </c>
       <c r="D25" s="5">
-        <v>0.019</v>
+        <v>1.9E-2</v>
       </c>
       <c r="E25" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>0</v>
@@ -1101,13 +1117,13 @@
         <v>1</v>
       </c>
       <c r="I25" s="4">
-        <v>0.335</v>
+        <v>0.33500000000000002</v>
       </c>
       <c r="J25" s="5">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="K25" s="4">
-        <v>0.145</v>
+        <v>0.14499999999999999</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>0</v>
@@ -1116,27 +1132,27 @@
         <v>1</v>
       </c>
       <c r="O25" s="4">
-        <v>0.349</v>
+        <v>0.34899999999999998</v>
       </c>
       <c r="P25" s="5">
-        <v>0.037</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="Q25" s="4">
-        <v>0.171</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17">
+        <v>0.17100000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B26" s="4">
-        <v>0.788</v>
+        <v>0.78800000000000003</v>
       </c>
       <c r="C26" s="4">
         <v>1</v>
       </c>
       <c r="D26" s="5">
-        <v>0.016</v>
+        <v>1.6E-2</v>
       </c>
       <c r="E26" s="4">
         <v>0.221</v>
@@ -1145,22 +1161,22 @@
         <v>1</v>
       </c>
       <c r="H26" s="4">
-        <v>0.335</v>
+        <v>0.33500000000000002</v>
       </c>
       <c r="I26" s="4">
         <v>1</v>
       </c>
       <c r="J26" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="K26" s="5">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="N26" s="4">
-        <v>0.349</v>
+        <v>0.34899999999999998</v>
       </c>
       <c r="O26" s="4">
         <v>1</v>
@@ -1169,18 +1185,18 @@
         <v>0.187</v>
       </c>
       <c r="Q26" s="5">
-        <v>0.036</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17">
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B27" s="5">
-        <v>0.019</v>
+        <v>1.9E-2</v>
       </c>
       <c r="C27" s="5">
-        <v>0.016</v>
+        <v>1.6E-2</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
@@ -1192,22 +1208,22 @@
         <v>2</v>
       </c>
       <c r="H27" s="5">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="I27" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="J27" s="4">
         <v>1</v>
       </c>
       <c r="K27" s="4">
-        <v>0.335</v>
+        <v>0.33500000000000002</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>2</v>
       </c>
       <c r="N27" s="5">
-        <v>0.037</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="O27" s="4">
         <v>0.187</v>
@@ -1219,12 +1235,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B28" s="4">
-        <v>0.285</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="C28" s="4">
         <v>0.221</v>
@@ -1239,13 +1255,13 @@
         <v>3</v>
       </c>
       <c r="H28" s="4">
-        <v>0.145</v>
+        <v>0.14499999999999999</v>
       </c>
       <c r="I28" s="5">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="J28" s="4">
-        <v>0.335</v>
+        <v>0.33500000000000002</v>
       </c>
       <c r="K28" s="4">
         <v>1</v>
@@ -1254,10 +1270,10 @@
         <v>3</v>
       </c>
       <c r="N28" s="4">
-        <v>0.171</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="O28" s="5">
-        <v>0.036</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="P28" s="5">
         <v>0</v>
@@ -1266,7 +1282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>4</v>
       </c>
@@ -1277,7 +1293,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:17">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>9</v>
       </c>
@@ -1288,7 +1304,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:17">
+    <row r="33" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -1299,7 +1315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:17">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>0</v>
       </c>
@@ -1337,7 +1353,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:17">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>0</v>
       </c>
@@ -1345,13 +1361,13 @@
         <v>1</v>
       </c>
       <c r="C35" s="4">
-        <v>0.668</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="D35" s="4">
-        <v>0.341</v>
+        <v>0.34100000000000003</v>
       </c>
       <c r="E35" s="4">
-        <v>0.668</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>0</v>
@@ -1360,13 +1376,13 @@
         <v>1</v>
       </c>
       <c r="I35" s="4">
-        <v>0.274</v>
+        <v>0.27400000000000002</v>
       </c>
       <c r="J35" s="4">
         <v>0.19</v>
       </c>
       <c r="K35" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>0</v>
@@ -1378,33 +1394,33 @@
         <v>0.246</v>
       </c>
       <c r="P35" s="4">
-        <v>0.392</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="Q35" s="5">
-        <v>0.049</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17">
+        <v>4.9000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B36" s="4">
-        <v>0.668</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="C36" s="4">
         <v>1</v>
       </c>
       <c r="D36" s="4">
-        <v>0.266</v>
+        <v>0.26600000000000001</v>
       </c>
       <c r="E36" s="4">
-        <v>0.482</v>
+        <v>0.48199999999999998</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>1</v>
       </c>
       <c r="H36" s="4">
-        <v>0.274</v>
+        <v>0.27400000000000002</v>
       </c>
       <c r="I36" s="4">
         <v>1</v>
@@ -1413,7 +1429,7 @@
         <v>0.748</v>
       </c>
       <c r="K36" s="5">
-        <v>0.051</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>1</v>
@@ -1425,27 +1441,27 @@
         <v>1</v>
       </c>
       <c r="P36" s="5">
-        <v>0.049</v>
+        <v>4.9000000000000002E-2</v>
       </c>
       <c r="Q36" s="4">
-        <v>0.392</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17">
+        <v>0.39200000000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B37" s="4">
-        <v>0.341</v>
+        <v>0.34100000000000003</v>
       </c>
       <c r="C37" s="4">
-        <v>0.266</v>
+        <v>0.26600000000000001</v>
       </c>
       <c r="D37" s="4">
         <v>1</v>
       </c>
       <c r="E37" s="4">
-        <v>0.482</v>
+        <v>0.48199999999999998</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>2</v>
@@ -1460,36 +1476,36 @@
         <v>1</v>
       </c>
       <c r="K37" s="4">
-        <v>0.078</v>
+        <v>7.8E-2</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>2</v>
       </c>
       <c r="N37" s="4">
-        <v>0.392</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="O37" s="5">
-        <v>0.049</v>
+        <v>4.9000000000000002E-2</v>
       </c>
       <c r="P37" s="4">
         <v>1</v>
       </c>
       <c r="Q37" s="5">
-        <v>0.008</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17">
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B38" s="4">
-        <v>0.668</v>
+        <v>0.66800000000000004</v>
       </c>
       <c r="C38" s="4">
-        <v>0.482</v>
+        <v>0.48199999999999998</v>
       </c>
       <c r="D38" s="4">
-        <v>0.482</v>
+        <v>0.48199999999999998</v>
       </c>
       <c r="E38" s="4">
         <v>1</v>
@@ -1498,13 +1514,13 @@
         <v>3</v>
       </c>
       <c r="H38" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="I38" s="5">
-        <v>0.051</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="J38" s="4">
-        <v>0.078</v>
+        <v>7.8E-2</v>
       </c>
       <c r="K38" s="4">
         <v>1</v>
@@ -1513,19 +1529,19 @@
         <v>3</v>
       </c>
       <c r="N38" s="5">
-        <v>0.049</v>
+        <v>4.9000000000000002E-2</v>
       </c>
       <c r="O38" s="4">
-        <v>0.392</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="P38" s="5">
-        <v>0.008</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="Q38" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:17">
+    <row r="41" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>4</v>
       </c>
@@ -1536,7 +1552,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="42" spans="1:17">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>10</v>
       </c>
@@ -1547,7 +1563,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:17">
+    <row r="43" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -1558,7 +1574,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:17">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>0</v>
       </c>
@@ -1596,7 +1612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:17">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>0</v>
       </c>
@@ -1607,10 +1623,10 @@
         <v>0.3</v>
       </c>
       <c r="D45" s="4">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="E45" s="4">
-        <v>0.978</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>0</v>
@@ -1619,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="I45" s="4">
-        <v>0.915</v>
+        <v>0.91500000000000004</v>
       </c>
       <c r="J45" s="4">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="K45" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>0</v>
@@ -1634,16 +1650,16 @@
         <v>1</v>
       </c>
       <c r="O45" s="4">
-        <v>0.239</v>
+        <v>0.23899999999999999</v>
       </c>
       <c r="P45" s="4">
         <v>0.108</v>
       </c>
       <c r="Q45" s="4">
-        <v>0.163</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17">
+        <v>0.16300000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>1</v>
       </c>
@@ -1654,7 +1670,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="4">
-        <v>0.763</v>
+        <v>0.76300000000000001</v>
       </c>
       <c r="E46" s="4">
         <v>0.3</v>
@@ -1663,63 +1679,63 @@
         <v>1</v>
       </c>
       <c r="H46" s="4">
-        <v>0.915</v>
+        <v>0.91500000000000004</v>
       </c>
       <c r="I46" s="4">
         <v>1</v>
       </c>
       <c r="J46" s="4">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="K46" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>1</v>
       </c>
       <c r="N46" s="4">
-        <v>0.239</v>
+        <v>0.23899999999999999</v>
       </c>
       <c r="O46" s="4">
         <v>1</v>
       </c>
       <c r="P46" s="4">
-        <v>0.521</v>
+        <v>0.52100000000000002</v>
       </c>
       <c r="Q46" s="5">
-        <v>0.012</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17">
+        <v>1.2E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B47" s="4">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="C47" s="4">
-        <v>0.763</v>
+        <v>0.76300000000000001</v>
       </c>
       <c r="D47" s="4">
         <v>1</v>
       </c>
       <c r="E47" s="4">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H47" s="4">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="I47" s="4">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="J47" s="4">
         <v>1</v>
       </c>
       <c r="K47" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>2</v>
@@ -1728,27 +1744,27 @@
         <v>0.108</v>
       </c>
       <c r="O47" s="4">
-        <v>0.521</v>
+        <v>0.52100000000000002</v>
       </c>
       <c r="P47" s="4">
         <v>1</v>
       </c>
       <c r="Q47" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B48" s="4">
-        <v>0.978</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="C48" s="4">
         <v>0.3</v>
       </c>
       <c r="D48" s="4">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="E48" s="4">
         <v>1</v>
@@ -1757,13 +1773,13 @@
         <v>3</v>
       </c>
       <c r="H48" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="I48" s="4">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="J48" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="K48" s="4">
         <v>1</v>
@@ -1772,13 +1788,13 @@
         <v>3</v>
       </c>
       <c r="N48" s="4">
-        <v>0.163</v>
+        <v>0.16300000000000001</v>
       </c>
       <c r="O48" s="5">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
       <c r="P48" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="Q48" s="4">
         <v>1</v>
@@ -1790,11 +1806,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1802,7 +1818,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
@@ -1810,7 +1826,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1818,7 +1834,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1844,7 +1860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1855,10 +1871,10 @@
         <v>1</v>
       </c>
       <c r="D5" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E5" s="4">
-        <v>0.765</v>
+        <v>0.76500000000000001</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>0</v>
@@ -1870,13 +1886,13 @@
         <v>0.2</v>
       </c>
       <c r="J5" s="5">
-        <v>0.014</v>
+        <v>1.4E-2</v>
       </c>
       <c r="K5" s="4">
-        <v>0.266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>0.26600000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
@@ -1887,10 +1903,10 @@
         <v>1</v>
       </c>
       <c r="D6" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E6" s="4">
-        <v>0.765</v>
+        <v>0.76500000000000001</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>1</v>
@@ -1905,30 +1921,30 @@
         <v>0.2</v>
       </c>
       <c r="K6" s="5">
-        <v>0.022</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>2.1999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="C7" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
       </c>
       <c r="E7" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H7" s="5">
-        <v>0.014</v>
+        <v>1.4E-2</v>
       </c>
       <c r="I7" s="4">
         <v>0.2</v>
@@ -1937,21 +1953,21 @@
         <v>1</v>
       </c>
       <c r="K7" s="5">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="4">
-        <v>0.765</v>
+        <v>0.76500000000000001</v>
       </c>
       <c r="C8" s="4">
-        <v>0.765</v>
+        <v>0.76500000000000001</v>
       </c>
       <c r="D8" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="E8" s="4">
         <v>1</v>
@@ -1960,19 +1976,19 @@
         <v>3</v>
       </c>
       <c r="H8" s="4">
-        <v>0.266</v>
+        <v>0.26600000000000001</v>
       </c>
       <c r="I8" s="5">
-        <v>0.022</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="J8" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="K8" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1980,7 +1996,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
@@ -1988,7 +2004,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -1996,7 +2012,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>0</v>
       </c>
@@ -2022,7 +2038,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>0</v>
       </c>
@@ -2033,10 +2049,10 @@
         <v>0.95</v>
       </c>
       <c r="D15" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E15" s="4">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>0</v>
@@ -2048,13 +2064,13 @@
         <v>0.214</v>
       </c>
       <c r="J15" s="4">
-        <v>0.142</v>
+        <v>0.14199999999999999</v>
       </c>
       <c r="K15" s="4">
         <v>0.15</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>1</v>
       </c>
@@ -2065,10 +2081,10 @@
         <v>1</v>
       </c>
       <c r="D16" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="E16" s="4">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>1</v>
@@ -2080,56 +2096,56 @@
         <v>1</v>
       </c>
       <c r="J16" s="4">
-        <v>0.647</v>
+        <v>0.64700000000000002</v>
       </c>
       <c r="K16" s="5">
-        <v>0.008</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B17" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="C17" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="D17" s="4">
         <v>1</v>
       </c>
       <c r="E17" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H17" s="4">
-        <v>0.142</v>
+        <v>0.14199999999999999</v>
       </c>
       <c r="I17" s="4">
-        <v>0.647</v>
+        <v>0.64700000000000002</v>
       </c>
       <c r="J17" s="4">
         <v>1</v>
       </c>
       <c r="K17" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B18" s="4">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="C18" s="4">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="D18" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="E18" s="4">
         <v>1</v>
@@ -2141,16 +2157,16 @@
         <v>0.15</v>
       </c>
       <c r="I18" s="5">
-        <v>0.008</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="J18" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="K18" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -2158,7 +2174,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -2166,7 +2182,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -2174,7 +2190,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>0</v>
       </c>
@@ -2200,7 +2216,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>0</v>
       </c>
@@ -2208,10 +2224,10 @@
         <v>1</v>
       </c>
       <c r="C25" s="4">
-        <v>0.416</v>
+        <v>0.41599999999999998</v>
       </c>
       <c r="D25" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="E25" s="4">
         <v>1</v>
@@ -2223,36 +2239,36 @@
         <v>1</v>
       </c>
       <c r="I25" s="4">
-        <v>0.338</v>
+        <v>0.33800000000000002</v>
       </c>
       <c r="J25" s="5">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="K25" s="4">
-        <v>0.362</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+        <v>0.36199999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B26" s="4">
-        <v>0.416</v>
+        <v>0.41599999999999998</v>
       </c>
       <c r="C26" s="4">
         <v>1</v>
       </c>
       <c r="D26" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="E26" s="4">
-        <v>0.416</v>
+        <v>0.41599999999999998</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="H26" s="4">
-        <v>0.338</v>
+        <v>0.33800000000000002</v>
       </c>
       <c r="I26" s="4">
         <v>1</v>
@@ -2261,30 +2277,30 @@
         <v>0.123</v>
       </c>
       <c r="K26" s="4">
-        <v>0.094</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B27" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="C27" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="D27" s="4">
         <v>1</v>
       </c>
       <c r="E27" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H27" s="5">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="I27" s="4">
         <v>0.123</v>
@@ -2293,10 +2309,10 @@
         <v>1</v>
       </c>
       <c r="K27" s="5">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
@@ -2304,10 +2320,10 @@
         <v>1</v>
       </c>
       <c r="C28" s="4">
-        <v>0.416</v>
+        <v>0.41599999999999998</v>
       </c>
       <c r="D28" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="E28" s="4">
         <v>1</v>
@@ -2316,19 +2332,19 @@
         <v>3</v>
       </c>
       <c r="H28" s="4">
-        <v>0.362</v>
+        <v>0.36199999999999999</v>
       </c>
       <c r="I28" s="4">
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="J28" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="K28" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>11</v>
       </c>
@@ -2336,7 +2352,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>25</v>
       </c>
@@ -2344,7 +2360,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -2352,7 +2368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>0</v>
       </c>
@@ -2378,7 +2394,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>0</v>
       </c>
@@ -2389,7 +2405,7 @@
         <v>1</v>
       </c>
       <c r="D35" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="E35" s="4">
         <v>1</v>
@@ -2401,16 +2417,16 @@
         <v>1</v>
       </c>
       <c r="I35" s="4">
-        <v>0.8149999999999999</v>
+        <v>0.81499999999999995</v>
       </c>
       <c r="J35" s="5">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="K35" s="4">
-        <v>0.536</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11">
+        <v>0.53600000000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>1</v>
       </c>
@@ -2421,7 +2437,7 @@
         <v>1</v>
       </c>
       <c r="D36" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="E36" s="4">
         <v>1</v>
@@ -2430,51 +2446,51 @@
         <v>1</v>
       </c>
       <c r="H36" s="4">
-        <v>0.8149999999999999</v>
+        <v>0.81499999999999995</v>
       </c>
       <c r="I36" s="4">
         <v>1</v>
       </c>
       <c r="J36" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="K36" s="4">
         <v>0.48</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B37" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="C37" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="D37" s="4">
         <v>1</v>
       </c>
       <c r="E37" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H37" s="5">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="I37" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="J37" s="4">
         <v>1</v>
       </c>
       <c r="K37" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
@@ -2485,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="D38" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="E38" s="4">
         <v>1</v>
@@ -2494,13 +2510,13 @@
         <v>3</v>
       </c>
       <c r="H38" s="4">
-        <v>0.536</v>
+        <v>0.53600000000000003</v>
       </c>
       <c r="I38" s="4">
         <v>0.48</v>
       </c>
       <c r="J38" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="K38" s="4">
         <v>1</v>

</xml_diff>